<commit_message>
Process Jeremy's latest workout entry
</commit_message>
<xml_diff>
--- a/Reports/Members/Jeremy_Activity_Report.xlsx
+++ b/Reports/Members/Jeremy_Activity_Report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -849,6 +849,53 @@
         </is>
       </c>
       <c r="I11" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>5/21/2026 18:56:16</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Jeremy</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Run/Jog</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2.88</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Strava</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
@@ -897,7 +944,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>26.57</v>
+        <v>29.45</v>
       </c>
       <c r="C2" t="n">
         <v>0</v>
@@ -967,7 +1014,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>44.1</v>
+        <v>46.98</v>
       </c>
       <c r="C6" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
fix: correct Kelvin's run distance, fix total points calculation bug, and fix Google Sheets CSV fallback URL
</commit_message>
<xml_diff>
--- a/Reports/Members/Jeremy_Activity_Report.xlsx
+++ b/Reports/Members/Jeremy_Activity_Report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1025,6 +1025,53 @@
       <c r="I13" t="inlineStr">
         <is>
           <t>Verified</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>6/3/2026 18:54:32</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Jeremy</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Run/Jog</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>7.24</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Strava</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Flagged</t>
         </is>
       </c>
     </row>
@@ -1071,13 +1118,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>73.69</v>
+        <v>80.93000000000001</v>
       </c>
       <c r="C2" t="n">
         <v>3390</v>
       </c>
       <c r="D2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -1141,13 +1188,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>73.69</v>
+        <v>80.93000000000001</v>
       </c>
       <c r="C6" t="n">
         <v>3390</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update: Week 24 new entries - Jeremy, Kelvin, Kai Fong (6/10)
</commit_message>
<xml_diff>
--- a/Reports/Members/Jeremy_Activity_Report.xlsx
+++ b/Reports/Members/Jeremy_Activity_Report.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1266,45 +1266,92 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>6/10/2026 18:07:46</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Jeremy</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Run/Jog</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>3.64</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Committee Approval Required</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>6/9/2026 18:31:22</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Jeremy</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>Run/Jog</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Jeremy</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Run/Jog</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
         <is>
           <t>7.05</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>Unknown</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>View</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
         <is>
           <t>Committee Approval Required</t>
         </is>
@@ -1353,13 +1400,13 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>117.23</v>
+        <v>120.87</v>
       </c>
       <c r="C2" t="n">
         <v>3390</v>
       </c>
       <c r="D2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3">
@@ -1423,13 +1470,13 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>117.23</v>
+        <v>120.87</v>
       </c>
       <c r="C6" t="n">
         <v>3390</v>
       </c>
       <c r="D6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
   </sheetData>

</xml_diff>